<commit_message>
new classes for load test
</commit_message>
<xml_diff>
--- a/src/test/resources/dataFile/testData.xlsx
+++ b/src/test/resources/dataFile/testData.xlsx
@@ -12,9 +12,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
   <si>
-    <t>?TSI=Test21</t>
+    <t>?TSI=Test38</t>
+  </si>
+  <si>
+    <t>?TSI=Test94</t>
+  </si>
+  <si>
+    <t>?TSI=Test17</t>
+  </si>
+  <si>
+    <t>?TSI=Test7</t>
+  </si>
+  <si>
+    <t>?TSI=Test32</t>
+  </si>
+  <si>
+    <t>?TSI=Test67</t>
+  </si>
+  <si>
+    <t>?TSI=Test3</t>
+  </si>
+  <si>
+    <t>?TSI=Test76</t>
   </si>
 </sst>
 </file>
@@ -59,12 +80,57 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="C3"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+    </row>
     <row r="3">
-      <c r="C3" t="s">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
         <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated testng test to handle both internal and uploaded fax numbers file
</commit_message>
<xml_diff>
--- a/src/test/resources/dataFile/testData.xlsx
+++ b/src/test/resources/dataFile/testData.xlsx
@@ -12,30 +12,36 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
-    <t>?TSI=Test805e700b</t>
+    <t>?TSI=Testbb4aed12</t>
   </si>
   <si>
-    <t>4392120277</t>
+    <t>2392120</t>
   </si>
   <si>
-    <t>?TSI=Testb039e82d</t>
+    <t>?TSI=Test23a51f6e</t>
   </si>
   <si>
-    <t>6392120277</t>
+    <t>83921</t>
   </si>
   <si>
-    <t>?TSI=Test0acb1772</t>
+    <t>?TSI=Test5d587460</t>
   </si>
   <si>
-    <t>9392120277</t>
+    <t>739212</t>
   </si>
   <si>
-    <t>?TSI=Test1ee1927f</t>
+    <t>?TSI=Testa57015ed</t>
   </si>
   <si>
-    <t>0116620479273</t>
+    <t>01166204</t>
+  </si>
+  <si>
+    <t>?TSI=Testd24ea860</t>
+  </si>
+  <si>
+    <t>63921</t>
   </si>
 </sst>
 </file>
@@ -80,7 +86,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -115,6 +121,14 @@
         <v>7</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
new regression test converted to smoke update
</commit_message>
<xml_diff>
--- a/src/test/resources/dataFile/testData.xlsx
+++ b/src/test/resources/dataFile/testData.xlsx
@@ -12,27 +12,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
   <si>
-    <t>?TSI=Test764914b2</t>
+    <t>?TSI=Test09b79555</t>
   </si>
   <si>
-    <t>83921</t>
+    <t>01166204</t>
   </si>
   <si>
-    <t>?TSI=Testa87d9e09</t>
+    <t>?TSI=Test4831b865</t>
   </si>
   <si>
-    <t>739212</t>
+    <t>2392120</t>
   </si>
   <si>
-    <t>?TSI=Test78cc7dcf</t>
+    <t>?TSI=Test6ea7e70a</t>
   </si>
   <si>
-    <t>?TSI=Teste280c981</t>
+    <t>?TSI=Test425ac7f6</t>
   </si>
   <si>
-    <t>?TSI=Test28d1312c</t>
+    <t>?TSI=Testa6995fa4</t>
+  </si>
+  <si>
+    <t>3392120</t>
   </si>
 </sst>
 </file>
@@ -117,7 +120,7 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
soap test body change commit
</commit_message>
<xml_diff>
--- a/src/test/resources/dataFile/testData.xlsx
+++ b/src/test/resources/dataFile/testData.xlsx
@@ -12,27 +12,57 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
-  <si>
-    <t>?TSI=Test09b79555</t>
-  </si>
-  <si>
-    <t>01166204</t>
-  </si>
-  <si>
-    <t>?TSI=Test4831b865</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
+  <si>
+    <t>?TSI=Test7d44176d</t>
+  </si>
+  <si>
+    <t>439212</t>
+  </si>
+  <si>
+    <t>?TSI=Testfc5dff19</t>
+  </si>
+  <si>
+    <t>739212</t>
+  </si>
+  <si>
+    <t>?TSI=Test236c6429</t>
+  </si>
+  <si>
+    <t>?TSI=Testf0f2a2ea</t>
   </si>
   <si>
     <t>2392120</t>
   </si>
   <si>
-    <t>?TSI=Test6ea7e70a</t>
-  </si>
-  <si>
-    <t>?TSI=Test425ac7f6</t>
-  </si>
-  <si>
-    <t>?TSI=Testa6995fa4</t>
+    <t>?TSI=Test94b9bee8</t>
+  </si>
+  <si>
+    <t>?TSI=Test5304454f</t>
+  </si>
+  <si>
+    <t>?TSI=Testc86dbe57</t>
+  </si>
+  <si>
+    <t>(222)34567</t>
+  </si>
+  <si>
+    <t>?TSI=Testdb42c3e9</t>
+  </si>
+  <si>
+    <t>?TSI=Testd6577016</t>
+  </si>
+  <si>
+    <t>abs234</t>
+  </si>
+  <si>
+    <t>?TSI=Test27b41686</t>
+  </si>
+  <si>
+    <t>?TSI=Testc93bd847</t>
+  </si>
+  <si>
+    <t>?TSI=Test80dba9b1</t>
   </si>
   <si>
     <t>3392120</t>
@@ -80,7 +110,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -104,7 +134,7 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -112,15 +142,71 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
         <v>6</v>
       </c>
-      <c r="B5" t="s">
-        <v>7</v>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new changes to json.data file test cases
</commit_message>
<xml_diff>
--- a/src/test/resources/dataFile/testData.xlsx
+++ b/src/test/resources/dataFile/testData.xlsx
@@ -14,10 +14,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
-    <t>?TSI=Test0a5f898f</t>
+    <t>?TSI=Test090b587a</t>
   </si>
   <si>
-    <t>(222)34567</t>
+    <t xml:space="preserve">   123</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Added new tests and udpated the pdf files
</commit_message>
<xml_diff>
--- a/src/test/resources/dataFile/testData.xlsx
+++ b/src/test/resources/dataFile/testData.xlsx
@@ -1,13 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25928"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\workspace\fs_test\src\test\resources\dataFile\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD5B39B6-BC3C-4B78-A529-3D2820C35F66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="4755" yWindow="1485" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="FIRST_SHEET" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,8 +24,12 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -330,7 +340,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>

</xml_diff>